<commit_message>
fixing rolling stock guangzhou line 7 data and all intersections have been examined
</commit_message>
<xml_diff>
--- a/deadline_energy_nsga2.xlsx
+++ b/deadline_energy_nsga2.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="21" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="33" uniqueCount="3">
   <si>
     <t>T_deadline_s</t>
   </si>
@@ -88,2750 +88,2748 @@
     </row>
     <row r="2">
       <c r="A2" s="0">
-        <v>129.50824179088957</v>
+        <v>189.92817092193403</v>
       </c>
       <c r="B2" s="0">
-        <v>23.161966706495619</v>
+        <v>71.919045447429113</v>
       </c>
       <c r="C2" s="0"/>
     </row>
     <row r="3">
       <c r="A3" s="0">
-        <v>130.0890881586692</v>
+        <v>190.56782276341153</v>
       </c>
       <c r="B3" s="0">
-        <v>20.627517848852104</v>
-      </c>
-      <c r="C3" s="0">
-        <v>20.564285584716753</v>
-      </c>
+        <v>71.812356013085847</v>
+      </c>
+      <c r="C3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="0">
-        <v>130.66993452644883</v>
+        <v>191.20747460488903</v>
       </c>
       <c r="B4" s="0">
-        <v>19.433264511847543</v>
+        <v>71.546730686183153</v>
       </c>
       <c r="C4" s="0">
-        <v>18.171564208201332</v>
+        <v>68.299225179782994</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0">
-        <v>131.25078089422848</v>
+        <v>191.84712644636653</v>
       </c>
       <c r="B5" s="0">
-        <v>18.551895727641284</v>
+        <v>70.918381629183017</v>
       </c>
       <c r="C5" s="0">
-        <v>16.837656324623058</v>
+        <v>66.925122531201339</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0">
-        <v>131.83162726200811</v>
+        <v>192.486778287844</v>
       </c>
       <c r="B6" s="0">
-        <v>17.670809233142045</v>
+        <v>70.352151865126785</v>
       </c>
       <c r="C6" s="0">
-        <v>16.060572740779659</v>
+        <v>66.073349981378243</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0">
-        <v>132.41247362978774</v>
+        <v>193.12643012932151</v>
       </c>
       <c r="B7" s="0">
-        <v>16.815986234707886</v>
+        <v>69.831652511819243</v>
       </c>
       <c r="C7" s="0">
-        <v>15.023439503102011</v>
+        <v>65.33280784999215</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0">
-        <v>132.99331999756737</v>
+        <v>193.76608197079901</v>
       </c>
       <c r="B8" s="0">
-        <v>16.098518520284664</v>
+        <v>69.619419951504227</v>
       </c>
       <c r="C8" s="0">
-        <v>14.360410028400704</v>
+        <v>64.752060972668303</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0">
-        <v>133.574166365347</v>
+        <v>194.40573381227651</v>
       </c>
       <c r="B9" s="0">
-        <v>15.189846665733956</v>
+        <v>69.325775141583478</v>
       </c>
       <c r="C9" s="0">
-        <v>13.759407969286423</v>
+        <v>67.34393896189134</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>134.15501273312665</v>
+        <v>195.04538565375401</v>
       </c>
       <c r="B10" s="0">
-        <v>14.290260231470398</v>
+        <v>68.756149625832435</v>
       </c>
       <c r="C10" s="0">
-        <v>13.27929416848853</v>
+        <v>65.842321715316516</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0">
-        <v>134.73585910090628</v>
+        <v>195.68503749523151</v>
       </c>
       <c r="B11" s="0">
-        <v>13.866207663184557</v>
+        <v>68.391732891963528</v>
       </c>
       <c r="C11" s="0">
-        <v>12.805006844034985</v>
+        <v>65.694733397570587</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0">
-        <v>135.31670546868591</v>
+        <v>196.32468933670899</v>
       </c>
       <c r="B12" s="0">
-        <v>12.516563435716423</v>
+        <v>68.176201023159621</v>
       </c>
       <c r="C12" s="0">
-        <v>12.363977287952681</v>
+        <v>64.537717512780461</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0">
-        <v>135.89755183646554</v>
+        <v>196.96434117818649</v>
       </c>
       <c r="B13" s="0">
-        <v>12.322000945852579</v>
+        <v>67.588779014564977</v>
       </c>
       <c r="C13" s="0">
-        <v>11.969592470690348</v>
+        <v>63.851464076732746</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0">
-        <v>136.47839820424517</v>
+        <v>197.60399301966399</v>
       </c>
       <c r="B14" s="0">
-        <v>12.115547703927815</v>
+        <v>67.335723330860887</v>
       </c>
       <c r="C14" s="0">
-        <v>11.632896399436722</v>
+        <v>63.596023034054497</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0">
-        <v>137.0592445720248</v>
+        <v>198.24364486114149</v>
       </c>
       <c r="B15" s="0">
-        <v>11.942663905592976</v>
+        <v>66.703007170441708</v>
       </c>
       <c r="C15" s="0">
-        <v>11.28013057370293</v>
+        <v>62.70564967858774</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0">
-        <v>137.64009093980445</v>
+        <v>198.88329670261899</v>
       </c>
       <c r="B16" s="0">
-        <v>11.220836171093648</v>
+        <v>66.473871539522463</v>
       </c>
       <c r="C16" s="0">
-        <v>11.003994148428824</v>
+        <v>62.142643406702632</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0">
-        <v>138.22093730758408</v>
+        <v>199.52294854409649</v>
       </c>
       <c r="B17" s="0">
-        <v>10.853933174375399</v>
+        <v>66.299909047750305</v>
       </c>
       <c r="C17" s="0">
-        <v>10.620494933790646</v>
+        <v>62.000687844931264</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0">
-        <v>138.80178367536371</v>
+        <v>200.162600385574</v>
       </c>
       <c r="B18" s="0">
-        <v>10.544492156988177</v>
+        <v>66.013052689490195</v>
       </c>
       <c r="C18" s="0">
-        <v>10.292161428719375</v>
+        <v>61.451752092922092</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0">
-        <v>139.38263004314334</v>
+        <v>200.80225222705147</v>
       </c>
       <c r="B19" s="0">
-        <v>10.30551904603843</v>
+        <v>65.686347381020184</v>
       </c>
       <c r="C19" s="0">
-        <v>9.9720887516718388</v>
+        <v>61.379790168614875</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0">
-        <v>139.96347641092296</v>
+        <v>201.44190406852897</v>
       </c>
       <c r="B20" s="0">
-        <v>9.9500951818265406</v>
+        <v>65.465401189820938</v>
       </c>
       <c r="C20" s="0">
-        <v>9.7440702996231607</v>
+        <v>60.69050946061094</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0">
-        <v>140.54432277870262</v>
+        <v>202.08155591000647</v>
       </c>
       <c r="B21" s="0">
-        <v>9.7145210738350052</v>
+        <v>64.793407272828574</v>
       </c>
       <c r="C21" s="0">
-        <v>9.4011580175578011</v>
+        <v>60.558806814272991</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0">
-        <v>141.12516914648225</v>
+        <v>202.72120775148397</v>
       </c>
       <c r="B22" s="0">
-        <v>9.5272363400219327</v>
+        <v>64.391851183906297</v>
       </c>
       <c r="C22" s="0">
-        <v>9.1111256208540326</v>
+        <v>60.339480936555859</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0">
-        <v>141.70601551426188</v>
+        <v>203.36085959296148</v>
       </c>
       <c r="B23" s="0">
-        <v>9.2700337613532167</v>
+        <v>64.16628505081971</v>
       </c>
       <c r="C23" s="0">
-        <v>8.8856913965505484</v>
+        <v>59.957354051540079</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0">
-        <v>142.28686188204151</v>
+        <v>204.00051143443898</v>
       </c>
       <c r="B24" s="0">
-        <v>9.0186654254651977</v>
+        <v>63.989562403750227</v>
       </c>
       <c r="C24" s="0">
-        <v>8.626336619914607</v>
+        <v>59.725352708126202</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0">
-        <v>142.86770824982114</v>
+        <v>204.64016327591645</v>
       </c>
       <c r="B25" s="0">
-        <v>8.7970550664969132</v>
+        <v>63.590978974862821</v>
       </c>
       <c r="C25" s="0">
-        <v>8.3930746609614104</v>
+        <v>59.48169200735201</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0">
-        <v>143.44855461760079</v>
+        <v>205.27981511739395</v>
       </c>
       <c r="B26" s="0">
-        <v>8.5942872714946201</v>
+        <v>63.570026173586044</v>
       </c>
       <c r="C26" s="0">
-        <v>8.1519254722468233</v>
+        <v>59.186494441403845</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0">
-        <v>144.02940098538042</v>
+        <v>205.91946695887145</v>
       </c>
       <c r="B27" s="0">
-        <v>8.2718510489547423</v>
+        <v>63.370303627883118</v>
       </c>
       <c r="C27" s="0">
-        <v>7.867955865184344</v>
+        <v>58.980803836138165</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0">
-        <v>144.61024735316005</v>
+        <v>206.55911880034896</v>
       </c>
       <c r="B28" s="0">
-        <v>7.8911840269930593</v>
+        <v>62.572669243151083</v>
       </c>
       <c r="C28" s="0">
-        <v>7.6483552004878188</v>
+        <v>58.793900268441561</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0">
-        <v>145.19109372093968</v>
+        <v>207.19877064182646</v>
       </c>
       <c r="B29" s="0">
-        <v>7.6143816171122394</v>
+        <v>62.3677756980588</v>
       </c>
       <c r="C29" s="0">
-        <v>7.4431214877619167</v>
+        <v>58.682275789907493</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0">
-        <v>145.7719400887193</v>
+        <v>207.83842248330396</v>
       </c>
       <c r="B30" s="0">
-        <v>7.3647616025368707</v>
+        <v>62.144219240241242</v>
       </c>
       <c r="C30" s="0">
-        <v>7.2285400881896145</v>
+        <v>58.352504756472428</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0">
-        <v>146.35278645649896</v>
+        <v>208.47807432478146</v>
       </c>
       <c r="B31" s="0">
-        <v>7.1070505521484932</v>
+        <v>61.920301655111601</v>
       </c>
       <c r="C31" s="0">
-        <v>7.0128009681368688</v>
+        <v>58.181001162864774</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0">
-        <v>146.93363282427859</v>
+        <v>209.11772616625893</v>
       </c>
       <c r="B32" s="0">
-        <v>6.8599091862315014</v>
+        <v>61.764269449351971</v>
       </c>
       <c r="C32" s="0">
-        <v>6.8742534903318591</v>
+        <v>57.984063840789027</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0">
-        <v>147.51447919205822</v>
+        <v>209.75737800773644</v>
       </c>
       <c r="B33" s="0">
-        <v>6.635120941015396</v>
+        <v>61.470023086600449</v>
       </c>
       <c r="C33" s="0">
-        <v>6.6011952796510673</v>
+        <v>57.769815821594001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0">
-        <v>148.09532555983785</v>
+        <v>210.39702984921394</v>
       </c>
       <c r="B34" s="0">
-        <v>6.4430178439905887</v>
+        <v>61.253697300905543</v>
       </c>
       <c r="C34" s="0">
-        <v>6.4084629144363383</v>
+        <v>57.737410054228207</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0">
-        <v>148.67617192761747</v>
+        <v>211.03668169069144</v>
       </c>
       <c r="B35" s="0">
-        <v>6.1802246704886326</v>
+        <v>61.101163679627867</v>
       </c>
       <c r="C35" s="0">
-        <v>6.2262931100740229</v>
+        <v>57.431671468318726</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0">
-        <v>149.25701829539713</v>
+        <v>211.67633353216894</v>
       </c>
       <c r="B36" s="0">
-        <v>6.1398327274075086</v>
+        <v>60.803548831690442</v>
       </c>
       <c r="C36" s="0">
-        <v>6.0085000877711039</v>
+        <v>57.294872796339405</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0">
-        <v>149.83786466317676</v>
+        <v>212.31598537364644</v>
       </c>
       <c r="B37" s="0">
-        <v>6.0474205552630043</v>
+        <v>60.69078058708179</v>
       </c>
       <c r="C37" s="0">
-        <v>5.8807590736155673</v>
+        <v>57.089393053981311</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0">
-        <v>150.41871103095639</v>
+        <v>212.95563721512394</v>
       </c>
       <c r="B38" s="0">
-        <v>5.6748268358180169</v>
+        <v>60.504568259928533</v>
       </c>
       <c r="C38" s="0">
-        <v>5.6810443728419653</v>
+        <v>56.835163887771344</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0">
-        <v>150.99955739873602</v>
+        <v>213.59528905660142</v>
       </c>
       <c r="B39" s="0">
-        <v>5.4835013380040998</v>
+        <v>60.193935601732278</v>
       </c>
       <c r="C39" s="0">
-        <v>5.4824229955816382</v>
+        <v>56.755679233991316</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0">
-        <v>151.58040376651565</v>
+        <v>214.23494089807892</v>
       </c>
       <c r="B40" s="0">
-        <v>5.3866506551807145</v>
+        <v>60.087939661575462</v>
       </c>
       <c r="C40" s="0">
-        <v>5.3329462251451663</v>
+        <v>56.494913259544454</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0">
-        <v>152.1612501342953</v>
+        <v>214.87459273955642</v>
       </c>
       <c r="B41" s="0">
-        <v>5.2884420105467474</v>
+        <v>60.026241221522426</v>
       </c>
       <c r="C41" s="0">
-        <v>5.1736865669695771</v>
+        <v>56.331572591170954</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0">
-        <v>152.74209650207493</v>
+        <v>215.51424458103392</v>
       </c>
       <c r="B42" s="0">
-        <v>5.2884420105467474</v>
+        <v>59.364461539239912</v>
       </c>
       <c r="C42" s="0">
-        <v>5.0012015270743397</v>
+        <v>56.15468031696367</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0">
-        <v>153.32294286985456</v>
+        <v>216.15389642251142</v>
       </c>
       <c r="B43" s="0">
-        <v>5.2884420105467474</v>
+        <v>59.245757706067543</v>
       </c>
       <c r="C43" s="0">
-        <v>4.9029049526554971</v>
+        <v>56.014226326791182</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0">
-        <v>153.90378923763419</v>
+        <v>216.79354826398893</v>
       </c>
       <c r="B44" s="0">
-        <v>5.2884420105467474</v>
+        <v>58.971454866356808</v>
       </c>
       <c r="C44" s="0">
-        <v>4.866332450111555</v>
+        <v>55.962307533990085</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0">
-        <v>154.48463560541382</v>
+        <v>217.43320010546643</v>
       </c>
       <c r="B45" s="0">
-        <v>5.2884420105467474</v>
+        <v>58.877332775479758</v>
       </c>
       <c r="C45" s="0">
-        <v>4.866332450111555</v>
+        <v>55.710738479663647</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="0">
-        <v>155.06548197319347</v>
+        <v>218.0728519469439</v>
       </c>
       <c r="B46" s="0">
-        <v>5.0170221698168964</v>
+        <v>58.763013817568648</v>
       </c>
       <c r="C46" s="0">
-        <v>4.866332450111555</v>
+        <v>55.630105865269414</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="0">
-        <v>155.6463283409731</v>
+        <v>218.7125037884214</v>
       </c>
       <c r="B47" s="0">
-        <v>5.0170221698168964</v>
+        <v>58.568196465903625</v>
       </c>
       <c r="C47" s="0">
-        <v>4.7232255918566564</v>
+        <v>55.604024203892742</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="0">
-        <v>156.22717470875273</v>
+        <v>219.3521556298989</v>
       </c>
       <c r="B48" s="0">
-        <v>4.9467264571677685</v>
+        <v>58.112986098891497</v>
       </c>
       <c r="C48" s="0">
-        <v>4.7232255918566564</v>
+        <v>55.228508343744181</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="0">
-        <v>156.80802107653236</v>
+        <v>219.99180747137641</v>
       </c>
       <c r="B49" s="0">
-        <v>4.9111710574647631</v>
+        <v>58.074797156024005</v>
       </c>
       <c r="C49" s="0">
-        <v>4.7232255918566564</v>
+        <v>55.100381908642063</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="0">
-        <v>157.38886744431198</v>
+        <v>220.63145931285391</v>
       </c>
       <c r="B50" s="0">
-        <v>4.9111710574647631</v>
+        <v>57.816571140385463</v>
       </c>
       <c r="C50" s="0">
-        <v>4.6409932725370986</v>
+        <v>55.065651346348361</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="0">
-        <v>157.96971381209164</v>
+        <v>221.27111115433138</v>
       </c>
       <c r="B51" s="0">
-        <v>4.8392005462041112</v>
+        <v>57.626885655669433</v>
       </c>
       <c r="C51" s="0">
-        <v>4.335364289153322</v>
+        <v>54.782454421903935</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="0">
-        <v>158.55056017987127</v>
+        <v>221.91076299580888</v>
       </c>
       <c r="B52" s="0">
-        <v>4.8392005462041112</v>
+        <v>57.42983934100134</v>
       </c>
       <c r="C52" s="0">
-        <v>4.2085102447195419</v>
+        <v>54.64969009219513</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="0">
-        <v>159.1314065476509</v>
+        <v>222.55041483728638</v>
       </c>
       <c r="B53" s="0">
-        <v>4.8392005462041112</v>
+        <v>57.301013937274263</v>
       </c>
       <c r="C53" s="0">
-        <v>4.2085102447195419</v>
+        <v>54.472232406718945</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="0">
-        <v>159.71225291543053</v>
+        <v>223.19006667876388</v>
       </c>
       <c r="B54" s="0">
-        <v>4.7289451815026933</v>
+        <v>57.039473656000396</v>
       </c>
       <c r="C54" s="0">
-        <v>4.1122868290447503</v>
+        <v>54.270797936363081</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="0">
-        <v>160.29309928321015</v>
+        <v>223.82971852024139</v>
       </c>
       <c r="B55" s="0">
-        <v>4.7289451815026933</v>
+        <v>56.849976327815739</v>
       </c>
       <c r="C55" s="0">
-        <v>4.1122868290447503</v>
+        <v>54.142388775919471</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="0">
-        <v>160.87394565098978</v>
+        <v>224.46937036171889</v>
       </c>
       <c r="B56" s="0">
-        <v>4.7289451815026933</v>
+        <v>56.707381219471969</v>
       </c>
       <c r="C56" s="0">
-        <v>4.0559768287919029</v>
+        <v>54.032633470892009</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="0">
-        <v>161.45479201876941</v>
+        <v>225.10902220319639</v>
       </c>
       <c r="B57" s="0">
-        <v>4.7289451815026933</v>
+        <v>56.639211796378774</v>
       </c>
       <c r="C57" s="0">
-        <v>4.0559768287919029</v>
+        <v>53.95079930001716</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="0">
-        <v>162.03563838654907</v>
+        <v>225.74867404467386</v>
       </c>
       <c r="B58" s="0">
-        <v>4.7289451815026933</v>
+        <v>56.415244534544712</v>
       </c>
       <c r="C58" s="0">
-        <v>3.9355676405332538</v>
+        <v>53.71317889477929</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="0">
-        <v>162.6164847543287</v>
+        <v>226.38832588615136</v>
       </c>
       <c r="B59" s="0">
-        <v>4.5771536214225224</v>
+        <v>56.178226354180836</v>
       </c>
       <c r="C59" s="0">
-        <v>3.9355676405332538</v>
+        <v>53.616980033339466</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="0">
-        <v>163.19733112210832</v>
+        <v>227.02797772762887</v>
       </c>
       <c r="B60" s="0">
-        <v>4.5382595433765207</v>
+        <v>56.024810511552474</v>
       </c>
       <c r="C60" s="0">
-        <v>3.9026558427590485</v>
+        <v>53.598649353856487</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="0">
-        <v>163.77817748988795</v>
+        <v>227.66762956910637</v>
       </c>
       <c r="B61" s="0">
-        <v>4.5382595433765207</v>
+        <v>55.647522928024216</v>
       </c>
       <c r="C61" s="0">
-        <v>3.9026558427590485</v>
+        <v>53.344795980356949</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="0">
-        <v>164.35902385766758</v>
+        <v>228.30728141058387</v>
       </c>
       <c r="B62" s="0">
-        <v>4.5382595433765207</v>
+        <v>55.458972793956569</v>
       </c>
       <c r="C62" s="0">
-        <v>3.9026558427590485</v>
+        <v>53.189871489622092</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="0">
-        <v>164.93987022544724</v>
+        <v>228.94693325206137</v>
       </c>
       <c r="B63" s="0">
-        <v>4.5382595433765207</v>
+        <v>55.371884905026413</v>
       </c>
       <c r="C63" s="0">
-        <v>3.9026558427590485</v>
+        <v>53.043711021445702</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="0">
-        <v>165.52071659322687</v>
+        <v>229.58658509353887</v>
       </c>
       <c r="B64" s="0">
-        <v>4.5382595433765207</v>
+        <v>55.126536539469626</v>
       </c>
       <c r="C64" s="0">
-        <v>3.9026558427590485</v>
+        <v>52.966135863856849</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="0">
-        <v>166.10156296100649</v>
+        <v>230.22623693501635</v>
       </c>
       <c r="B65" s="0">
-        <v>4.4190873502398178</v>
+        <v>55.064682525746498</v>
       </c>
       <c r="C65" s="0">
-        <v>3.9026558427590485</v>
+        <v>52.944634931281314</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="0">
-        <v>166.68240932878612</v>
+        <v>230.86588877649385</v>
       </c>
       <c r="B66" s="0">
-        <v>4.3789533497130861</v>
+        <v>55.022336769203811</v>
       </c>
       <c r="C66" s="0">
-        <v>3.569456315954894</v>
+        <v>52.660953032119821</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="0">
-        <v>167.26325569656575</v>
+        <v>231.50554061797135</v>
       </c>
       <c r="B67" s="0">
-        <v>4.3388193491863545</v>
+        <v>54.917048642449537</v>
       </c>
       <c r="C67" s="0">
-        <v>3.569456315954894</v>
+        <v>52.636999946243854</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="0">
-        <v>167.84410206434541</v>
+        <v>232.14519245944885</v>
       </c>
       <c r="B68" s="0">
-        <v>4.3388193491863545</v>
+        <v>54.666182507769207</v>
       </c>
       <c r="C68" s="0">
-        <v>3.569456315954894</v>
+        <v>52.449258725915648</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="0">
-        <v>168.42494843212503</v>
+        <v>232.78484430092635</v>
       </c>
       <c r="B69" s="0">
-        <v>4.2986853486596228</v>
+        <v>54.666182507769207</v>
       </c>
       <c r="C69" s="0">
-        <v>3.569456315954894</v>
+        <v>52.370338503789327</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="0">
-        <v>169.00579479990466</v>
+        <v>233.42449614240385</v>
       </c>
       <c r="B70" s="0">
-        <v>4.2986853486596228</v>
+        <v>54.5098166291734</v>
       </c>
       <c r="C70" s="0">
-        <v>3.569456315954894</v>
+        <v>52.193462107220555</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="0">
-        <v>169.58664116768432</v>
+        <v>234.06414798388136</v>
       </c>
       <c r="B71" s="0">
-        <v>4.2585513481328912</v>
+        <v>54.475327374334285</v>
       </c>
       <c r="C71" s="0">
-        <v>3.569456315954894</v>
+        <v>52.117346187008522</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="0">
-        <v>170.16748753546392</v>
+        <v>234.70379982535883</v>
       </c>
       <c r="B72" s="0">
-        <v>4.2184173476061595</v>
+        <v>54.385178507509849</v>
       </c>
       <c r="C72" s="0">
-        <v>3.569456315954894</v>
+        <v>51.995194423108728</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="0">
-        <v>170.74833390324358</v>
+        <v>235.34345166683633</v>
       </c>
       <c r="B73" s="0">
-        <v>4.2184173476061595</v>
+        <v>54.124222025871312</v>
       </c>
       <c r="C73" s="0">
-        <v>3.569456315954894</v>
+        <v>51.899406610275989</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="0">
-        <v>171.3291802710232</v>
+        <v>235.98310350831383</v>
       </c>
       <c r="B74" s="0">
-        <v>4.1782833470794278</v>
+        <v>53.980121431268593</v>
       </c>
       <c r="C74" s="0">
-        <v>3.3719347299476841</v>
+        <v>51.899406610275989</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="0">
-        <v>171.91002663880283</v>
+        <v>236.62275534979133</v>
       </c>
       <c r="B75" s="0">
-        <v>4.1782833470794278</v>
+        <v>53.886768457050707</v>
       </c>
       <c r="C75" s="0">
-        <v>3.3719347299476841</v>
+        <v>51.76571092700479</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="0">
-        <v>172.49087300658246</v>
+        <v>237.26240719126884</v>
       </c>
       <c r="B76" s="0">
-        <v>4.1381493465526962</v>
+        <v>53.697873573310218</v>
       </c>
       <c r="C76" s="0">
-        <v>3.3109049598215505</v>
+        <v>51.499495542216621</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="0">
-        <v>173.07171937436209</v>
+        <v>237.90205903274631</v>
       </c>
       <c r="B77" s="0">
-        <v>4.0980153460259645</v>
+        <v>53.529957046134811</v>
       </c>
       <c r="C77" s="0">
-        <v>2.860196168792239</v>
+        <v>51.373335292900862</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="0">
-        <v>173.65256574214175</v>
+        <v>238.54171087422381</v>
       </c>
       <c r="B78" s="0">
-        <v>4.0980153460259645</v>
+        <v>53.43551231414655</v>
       </c>
       <c r="C78" s="0">
-        <v>2.860196168792239</v>
+        <v>51.244218411494558</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="0">
-        <v>174.23341210992138</v>
+        <v>239.18136271570131</v>
       </c>
       <c r="B79" s="0">
-        <v>2.7692460363444829</v>
+        <v>53.40271990924758</v>
       </c>
       <c r="C79" s="0">
-        <v>2.860196168792239</v>
+        <v>51.219594878642255</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="0">
-        <v>174.814258477701</v>
+        <v>239.82101455717881</v>
       </c>
       <c r="B80" s="0">
-        <v>2.7692460363444829</v>
+        <v>53.212682045255626</v>
       </c>
       <c r="C80" s="0">
-        <v>2.860196168792239</v>
+        <v>51.05330089344794</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="0">
-        <v>175.39510484548063</v>
+        <v>240.46066639865632</v>
       </c>
       <c r="B81" s="0">
-        <v>2.7291120358177512</v>
+        <v>53.212682045255626</v>
       </c>
       <c r="C81" s="0">
-        <v>2.860196168792239</v>
+        <v>50.924475707299237</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="0">
-        <v>175.97595121326026</v>
+        <v>241.10031824013382</v>
       </c>
       <c r="B82" s="0">
-        <v>2.7291120358177512</v>
+        <v>52.947906570554835</v>
       </c>
       <c r="C82" s="0">
-        <v>2.860196168792239</v>
+        <v>50.858158535501929</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="0">
-        <v>176.55679758103992</v>
+        <v>241.73997008161132</v>
       </c>
       <c r="B83" s="0">
-        <v>2.5685760337108246</v>
+        <v>52.774969278484086</v>
       </c>
       <c r="C83" s="0">
-        <v>2.753206841441231</v>
+        <v>50.707217428972619</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="0">
-        <v>177.13764394881955</v>
+        <v>242.37962192308879</v>
       </c>
       <c r="B84" s="0">
-        <v>2.5685760337108246</v>
+        <v>52.671500714501235</v>
       </c>
       <c r="C84" s="0">
-        <v>2.753206841441231</v>
+        <v>50.669125936441738</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="0">
-        <v>177.71849031659917</v>
+        <v>243.01927376456632</v>
       </c>
       <c r="B85" s="0">
-        <v>2.4883080326573617</v>
+        <v>52.576148947527543</v>
       </c>
       <c r="C85" s="0">
-        <v>2.5885189386216885</v>
+        <v>50.528138246159031</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="0">
-        <v>178.2993366843788</v>
+        <v>243.6589256060438</v>
       </c>
       <c r="B86" s="0">
-        <v>2.4883080326573617</v>
+        <v>52.350083551567472</v>
       </c>
       <c r="C86" s="0">
-        <v>2.5885189386216885</v>
+        <v>50.413497612360899</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="0">
-        <v>178.88018305215843</v>
+        <v>244.2985774475213</v>
       </c>
       <c r="B87" s="0">
-        <v>2.4080400316038979</v>
+        <v>52.153314794459476</v>
       </c>
       <c r="C87" s="0">
-        <v>2.5885189386216885</v>
+        <v>50.342635895624</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="0">
-        <v>179.46102941993809</v>
+        <v>244.9382292889988</v>
       </c>
       <c r="B88" s="0">
-        <v>2.4080400316038979</v>
+        <v>52.056889206723866</v>
       </c>
       <c r="C88" s="0">
-        <v>2.5142968997837478</v>
+        <v>50.198969088000744</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="0">
-        <v>180.04187578771772</v>
+        <v>245.57788113047627</v>
       </c>
       <c r="B89" s="0">
-        <v>2.3679060310771663</v>
+        <v>51.965830258968374</v>
       </c>
       <c r="C89" s="0">
-        <v>2.5142968997837478</v>
+        <v>50.153883624426541</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="0">
-        <v>180.62272215549734</v>
+        <v>246.2175329719538</v>
       </c>
       <c r="B90" s="0">
-        <v>2.3679060310771663</v>
+        <v>51.827529930946838</v>
       </c>
       <c r="C90" s="0">
-        <v>2.5142968997837478</v>
+        <v>50.012760491229386</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="0">
-        <v>181.20356852327697</v>
+        <v>246.85718481343127</v>
       </c>
       <c r="B91" s="0">
-        <v>2.3679060310771663</v>
+        <v>51.755229916533438</v>
       </c>
       <c r="C91" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.905995725547278</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="0">
-        <v>181.7844148910566</v>
+        <v>247.49683665490878</v>
       </c>
       <c r="B92" s="0">
-        <v>2.3679060310771663</v>
+        <v>51.688940663007671</v>
       </c>
       <c r="C92" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.784470712904096</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="0">
-        <v>182.36526125883626</v>
+        <v>248.13648849638628</v>
       </c>
       <c r="B93" s="0">
-        <v>2.1672360284435079</v>
+        <v>51.455302047535611</v>
       </c>
       <c r="C93" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.716097622085542</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="0">
-        <v>182.94610762661588</v>
+        <v>248.77614033786378</v>
       </c>
       <c r="B94" s="0">
-        <v>2.1672360284435079</v>
+        <v>51.438214674609228</v>
       </c>
       <c r="C94" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.524280084729085</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="0">
-        <v>183.52695399439551</v>
+        <v>249.41579217934128</v>
       </c>
       <c r="B95" s="0">
-        <v>2.1271020279167763</v>
+        <v>51.231307555805451</v>
       </c>
       <c r="C95" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.501279917031411</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="0">
-        <v>184.10780036217514</v>
+        <v>250.05544402081878</v>
       </c>
       <c r="B96" s="0">
-        <v>2.1271020279167763</v>
+        <v>51.194078289906244</v>
       </c>
       <c r="C96" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.391816641959366</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="0">
-        <v>184.68864672995477</v>
+        <v>250.69509586229629</v>
       </c>
       <c r="B97" s="0">
-        <v>2.1271020279167763</v>
+        <v>51.1519191030944</v>
       </c>
       <c r="C97" s="0">
-        <v>2.2403015532874138</v>
+        <v>49.286839240141141</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="0">
-        <v>185.26949309773443</v>
+        <v>251.33474770377376</v>
       </c>
       <c r="B98" s="0">
-        <v>2.0067000263365813</v>
+        <v>51.055899114230968</v>
       </c>
       <c r="C98" s="0">
-        <v>2.1198995517072188</v>
+        <v>49.264681301011862</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="0">
-        <v>185.85033946551405</v>
+        <v>251.97439954525126</v>
       </c>
       <c r="B99" s="0">
-        <v>2.0067000263365813</v>
+        <v>50.992931714832267</v>
       </c>
       <c r="C99" s="0">
-        <v>2.0196142864204791</v>
+        <v>49.141611753534221</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="0">
-        <v>186.43118583329368</v>
+        <v>252.61405138672876</v>
       </c>
       <c r="B100" s="0">
-        <v>1.9665660258098496</v>
+        <v>50.992931714832267</v>
       </c>
       <c r="C100" s="0">
-        <v>2.0196142864204791</v>
+        <v>48.989479475693102</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="0">
-        <v>187.01203220107331</v>
+        <v>253.25370322820626</v>
       </c>
       <c r="B101" s="0">
-        <v>1.9665660258098496</v>
+        <v>50.808973356156926</v>
       </c>
       <c r="C101" s="0">
-        <v>2.0196142864204791</v>
+        <v>48.908582075598858</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="0">
-        <v>187.59287856885294</v>
+        <v>253.89335506968377</v>
       </c>
       <c r="B102" s="0">
-        <v>1.9665660258098496</v>
+        <v>50.620887592363722</v>
       </c>
       <c r="C102" s="0">
-        <v>2.0054257286503807</v>
+        <v>48.858645482818552</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="0">
-        <v>188.1737249366326</v>
+        <v>254.53300691116124</v>
       </c>
       <c r="B103" s="0">
-        <v>1.8862980247563865</v>
+        <v>50.620887592363722</v>
       </c>
       <c r="C103" s="0">
-        <v>2.0054257286503807</v>
+        <v>48.766626951183071</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="0">
-        <v>188.75457130441222</v>
+        <v>255.17265875263877</v>
       </c>
       <c r="B104" s="0">
-        <v>1.8862980247563865</v>
+        <v>50.541187800181888</v>
       </c>
       <c r="C104" s="0">
-        <v>2.0054257286503807</v>
+        <v>48.651430958476219</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="0">
-        <v>189.33541767219185</v>
+        <v>255.81231059411624</v>
       </c>
       <c r="B105" s="0">
-        <v>1.8461640242296549</v>
+        <v>50.495827565056175</v>
       </c>
       <c r="C105" s="0">
-        <v>2.0054257286503807</v>
+        <v>48.597571744553306</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="0">
-        <v>189.91626403997148</v>
+        <v>256.45196243559377</v>
       </c>
       <c r="B106" s="0">
-        <v>1.7658960231761913</v>
+        <v>50.202173834078309</v>
       </c>
       <c r="C106" s="0">
-        <v>2.0054257286503807</v>
+        <v>48.488405100398793</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="0">
-        <v>190.49711040775111</v>
+        <v>257.09161427707124</v>
       </c>
       <c r="B107" s="0">
-        <v>1.7658960231761913</v>
+        <v>50.183262379605985</v>
       </c>
       <c r="C107" s="0">
-        <v>1.8783912104323779</v>
+        <v>48.461156265262517</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="0">
-        <v>191.07795677553077</v>
+        <v>257.73126611854877</v>
       </c>
       <c r="B108" s="0">
-        <v>1.7257620226494597</v>
+        <v>50.112620028968621</v>
       </c>
       <c r="C108" s="0">
-        <v>1.8783912104323779</v>
+        <v>48.333630213969528</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="0">
-        <v>191.65880314331037</v>
+        <v>258.37091796002625</v>
       </c>
       <c r="B109" s="0">
-        <v>1.6856280221227282</v>
+        <v>50.072191481014357</v>
       </c>
       <c r="C109" s="0">
-        <v>1.8783912104323779</v>
+        <v>48.231499580906366</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="0">
-        <v>192.23964951109002</v>
+        <v>259.01056980150372</v>
       </c>
       <c r="B110" s="0">
-        <v>1.6856280221227282</v>
+        <v>49.989835566270358</v>
       </c>
       <c r="C110" s="0">
-        <v>1.8783912104323779</v>
+        <v>48.11361210167955</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="0">
-        <v>192.82049587886965</v>
+        <v>259.65022164298125</v>
       </c>
       <c r="B111" s="0">
-        <v>1.6454940215959968</v>
+        <v>49.907679515638648</v>
       </c>
       <c r="C111" s="0">
-        <v>1.8783912104323779</v>
+        <v>48.049517371465726</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="0">
-        <v>193.40134224664928</v>
+        <v>260.28987348445872</v>
       </c>
       <c r="B112" s="0">
-        <v>1.6454940215959968</v>
+        <v>49.759757330032755</v>
       </c>
       <c r="C112" s="0">
-        <v>1.8783912104323779</v>
+        <v>48.016907965285554</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="0">
-        <v>193.98218861442894</v>
+        <v>260.9295253259362</v>
       </c>
       <c r="B113" s="0">
-        <v>1.6454940215959968</v>
+        <v>49.599520289378361</v>
       </c>
       <c r="C113" s="0">
-        <v>1.8783912104323779</v>
+        <v>47.983041416044429</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="0">
-        <v>194.56303498220854</v>
+        <v>261.56917716741373</v>
       </c>
       <c r="B114" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.542198792227495</v>
       </c>
       <c r="C114" s="0">
-        <v>1.8783912104323779</v>
+        <v>47.983041416044429</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="0">
-        <v>195.14388134998819</v>
+        <v>262.20882900889126</v>
       </c>
       <c r="B115" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.425561312006742</v>
       </c>
       <c r="C115" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.720458941496105</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="0">
-        <v>195.72472771776782</v>
+        <v>262.84848085036873</v>
       </c>
       <c r="B116" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.403635573064683</v>
       </c>
       <c r="C116" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.692063015647335</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="0">
-        <v>196.30557408554745</v>
+        <v>263.4881326918462</v>
       </c>
       <c r="B117" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.359467608483911</v>
       </c>
       <c r="C117" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.555017092574048</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="0">
-        <v>196.8864204533271</v>
+        <v>264.12778453332373</v>
       </c>
       <c r="B118" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.199817738016208</v>
       </c>
       <c r="C118" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.555017092574048</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="0">
-        <v>197.46726682110671</v>
+        <v>264.76743637480121</v>
       </c>
       <c r="B119" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.159364835918794</v>
       </c>
       <c r="C119" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.388745174454968</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="0">
-        <v>198.04811318888636</v>
+        <v>265.40708821627868</v>
       </c>
       <c r="B120" s="0">
-        <v>1.6053600210692651</v>
+        <v>49.058799520542955</v>
       </c>
       <c r="C120" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.31057983891575</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="0">
-        <v>198.62895955666599</v>
+        <v>266.04674005775621</v>
       </c>
       <c r="B121" s="0">
-        <v>1.6053600210692651</v>
+        <v>48.96234417814523</v>
       </c>
       <c r="C121" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.238778544515455</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="0">
-        <v>199.20980592444562</v>
+        <v>266.68639189923368</v>
       </c>
       <c r="B122" s="0">
-        <v>1.6053600210692651</v>
+        <v>48.876651910563908</v>
       </c>
       <c r="C122" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.168629622082712</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="0">
-        <v>199.79065229222528</v>
+        <v>267.32604374071121</v>
       </c>
       <c r="B123" s="0">
-        <v>1.6053600210692651</v>
+        <v>48.825161449875267</v>
       </c>
       <c r="C123" s="0">
-        <v>1.7658960231761916</v>
+        <v>47.105145795802031</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="0">
-        <v>200.37149866000487</v>
+        <v>267.96569558218869</v>
       </c>
       <c r="B124" s="0">
-        <v>1.6053600210692651</v>
+        <v>48.665005309601916</v>
       </c>
       <c r="C124" s="0">
-        <v>1.468300794626761</v>
+        <v>47.105145795802031</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="0">
-        <v>200.95234502778453</v>
+        <v>268.60534742366622</v>
       </c>
       <c r="B125" s="0">
-        <v>1.6053600210692651</v>
+        <v>48.649963741467282</v>
       </c>
       <c r="C125" s="0">
-        <v>1.468300794626761</v>
+        <v>47.003161964791104</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="0">
-        <v>201.53319139556416</v>
+        <v>269.24499926514369</v>
       </c>
       <c r="B126" s="0">
-        <v>1.6053600210692651</v>
+        <v>48.582239858873663</v>
       </c>
       <c r="C126" s="0">
-        <v>1.468300794626761</v>
+        <v>46.904219463782539</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="0">
-        <v>202.11403776334379</v>
+        <v>269.88465110662116</v>
       </c>
       <c r="B127" s="0">
-        <v>1.4448240189623385</v>
+        <v>48.582239858873663</v>
       </c>
       <c r="C127" s="0">
-        <v>1.468300794626761</v>
+        <v>46.835881880232435</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="0">
-        <v>202.69488413112342</v>
+        <v>270.52430294809869</v>
       </c>
       <c r="B128" s="0">
-        <v>1.4448240189623385</v>
+        <v>48.493234527420555</v>
       </c>
       <c r="C128" s="0">
-        <v>1.468300794626761</v>
+        <v>46.835881880232435</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="0">
-        <v>203.27573049890304</v>
+        <v>271.16395478957617</v>
       </c>
       <c r="B129" s="0">
-        <v>1.4448240189623385</v>
+        <v>48.322213329202881</v>
       </c>
       <c r="C129" s="0">
-        <v>1.468300794626761</v>
+        <v>46.675895344018386</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="0">
-        <v>203.8565768666827</v>
+        <v>271.8036066310537</v>
       </c>
       <c r="B130" s="0">
-        <v>1.4448240189623385</v>
+        <v>48.23549962177372</v>
       </c>
       <c r="C130" s="0">
-        <v>1.468300794626761</v>
+        <v>46.591602826751967</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="0">
-        <v>204.4374232344623</v>
+        <v>272.44325847253117</v>
       </c>
       <c r="B131" s="0">
-        <v>1.4046900184356068</v>
+        <v>48.135366650041149</v>
       </c>
       <c r="C131" s="0">
-        <v>1.468300794626761</v>
+        <v>46.52081471195828</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="0">
-        <v>205.01826960224196</v>
+        <v>273.0829103140087</v>
       </c>
       <c r="B132" s="0">
-        <v>1.4046900184356068</v>
+        <v>48.049166330233028</v>
       </c>
       <c r="C132" s="0">
-        <v>1.468300794626761</v>
+        <v>46.431567195323495</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="0">
-        <v>205.59911597002159</v>
+        <v>273.72256215548617</v>
       </c>
       <c r="B133" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.959037941526574</v>
       </c>
       <c r="C133" s="0">
-        <v>1.468300794626761</v>
+        <v>46.322751886708872</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="0">
-        <v>206.17996233780122</v>
+        <v>274.36221399696365</v>
       </c>
       <c r="B134" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.941456294341883</v>
       </c>
       <c r="C134" s="0">
-        <v>1.1660249011683561</v>
+        <v>46.245791359770252</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="0">
-        <v>206.76080870558087</v>
+        <v>275.00186583844118</v>
       </c>
       <c r="B135" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.883865667685015</v>
       </c>
       <c r="C135" s="0">
-        <v>1.1660249011683561</v>
+        <v>46.212724585874305</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="0">
-        <v>207.3416550733605</v>
+        <v>275.64151767991865</v>
       </c>
       <c r="B136" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.883865667685015</v>
       </c>
       <c r="C136" s="0">
-        <v>1.1660249011683561</v>
+        <v>46.135106977911114</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="0">
-        <v>207.92250144114013</v>
+        <v>276.28116952139618</v>
       </c>
       <c r="B137" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.698845741433573</v>
       </c>
       <c r="C137" s="0">
-        <v>1.1660249011683561</v>
+        <v>46.135106977911114</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="0">
-        <v>208.50334780891978</v>
+        <v>276.92082136287365</v>
       </c>
       <c r="B138" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.62622500843284</v>
       </c>
       <c r="C138" s="0">
-        <v>1.1660249011683561</v>
+        <v>45.981612064132918</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="0">
-        <v>209.08419417669939</v>
+        <v>277.56047320435118</v>
       </c>
       <c r="B139" s="0">
-        <v>1.4046900184356068</v>
+        <v>47.585621045825853</v>
       </c>
       <c r="C139" s="0">
-        <v>1.1660249011683561</v>
+        <v>45.95817076215063</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="0">
-        <v>209.66504054447904</v>
+        <v>278.20012504582866</v>
       </c>
       <c r="B140" s="0">
-        <v>1.3244220173821435</v>
+        <v>47.554168465005738</v>
       </c>
       <c r="C140" s="0">
-        <v>1.088283093330189</v>
+        <v>45.835494024137688</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="0">
-        <v>210.24588691225867</v>
+        <v>278.83977688730613</v>
       </c>
       <c r="B141" s="0">
-        <v>1.3244220173821435</v>
+        <v>47.452309615076366</v>
       </c>
       <c r="C141" s="0">
-        <v>1.088283093330189</v>
+        <v>45.835494024137688</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="0">
-        <v>210.8267332800383</v>
+        <v>279.47942872878366</v>
       </c>
       <c r="B142" s="0">
-        <v>1.3244220173821435</v>
+        <v>47.452309615076366</v>
       </c>
       <c r="C142" s="0">
-        <v>1.088283093330189</v>
+        <v>45.698637993719089</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="0">
-        <v>211.40757964781795</v>
+        <v>280.11908057026113</v>
       </c>
       <c r="B143" s="0">
-        <v>1.3244220173821435</v>
+        <v>47.293309350403661</v>
       </c>
       <c r="C143" s="0">
-        <v>1.088283093330189</v>
+        <v>45.644369529716371</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="0">
-        <v>211.98842601559755</v>
+        <v>280.75873241173861</v>
       </c>
       <c r="B144" s="0">
-        <v>1.2842880168554118</v>
+        <v>47.217338357760667</v>
       </c>
       <c r="C144" s="0">
-        <v>1.088283093330189</v>
+        <v>45.628860134169145</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="0">
-        <v>212.56927238337721</v>
+        <v>281.39838425321614</v>
       </c>
       <c r="B145" s="0">
-        <v>1.2842880168554118</v>
+        <v>47.097197183797185</v>
       </c>
       <c r="C145" s="0">
-        <v>1.0629957329266191</v>
+        <v>45.548339169824487</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="0">
-        <v>213.15011875115684</v>
+        <v>282.03803609469367</v>
       </c>
       <c r="B146" s="0">
-        <v>1.2842880168554118</v>
+        <v>47.066616993920356</v>
       </c>
       <c r="C146" s="0">
-        <v>1.0629957329266191</v>
+        <v>45.494988036837988</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="0">
-        <v>213.73096511893647</v>
+        <v>282.67768793617114</v>
       </c>
       <c r="B147" s="0">
-        <v>1.2842880168554118</v>
+        <v>46.998712280954564</v>
       </c>
       <c r="C147" s="0">
-        <v>1.0629957329266191</v>
+        <v>45.494988036837988</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="0">
-        <v>214.3118114867161</v>
+        <v>283.31733977764861</v>
       </c>
       <c r="B148" s="0">
-        <v>1.2842880168554118</v>
+        <v>46.983969237614048</v>
       </c>
       <c r="C148" s="0">
-        <v>1.0372278870125571</v>
+        <v>45.33681333695057</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="0">
-        <v>214.89265785449572</v>
+        <v>283.95699161912614</v>
       </c>
       <c r="B149" s="0">
-        <v>1.2842880168554118</v>
+        <v>46.833951962020592</v>
       </c>
       <c r="C149" s="0">
-        <v>0.89348167075665685</v>
+        <v>45.286790246852547</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="0">
-        <v>215.47350422227538</v>
+        <v>284.59664346060362</v>
       </c>
       <c r="B150" s="0">
-        <v>1.2441540163286804</v>
+        <v>46.810743550792729</v>
       </c>
       <c r="C150" s="0">
-        <v>0.89348167075665685</v>
+        <v>45.231098383893311</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="0">
-        <v>216.05435059005498</v>
+        <v>285.23629530208115</v>
       </c>
       <c r="B151" s="0">
-        <v>1.2441540163286804</v>
+        <v>46.716860175884662</v>
       </c>
       <c r="C151" s="0">
-        <v>0.89348167075665685</v>
+        <v>45.158455080428695</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="0">
-        <v>216.63519695783464</v>
+        <v>285.87594714355862</v>
       </c>
       <c r="B152" s="0">
-        <v>1.2441540163286804</v>
+        <v>46.67415449930985</v>
       </c>
       <c r="C152" s="0">
-        <v>0.89348167075665685</v>
+        <v>45.103177912447379</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="0">
-        <v>217.21604332561427</v>
+        <v>286.51559898503615</v>
       </c>
       <c r="B153" s="0">
-        <v>1.2441540163286804</v>
+        <v>46.548126039307945</v>
       </c>
       <c r="C153" s="0">
-        <v>0.89348167075665685</v>
+        <v>45.029477188044311</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="0">
-        <v>217.79688969339389</v>
+        <v>287.15525082651362</v>
       </c>
       <c r="B154" s="0">
-        <v>1.2441540163286804</v>
+        <v>46.474177831930916</v>
       </c>
       <c r="C154" s="0">
-        <v>0.89348167075665685</v>
+        <v>45.029477188044311</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="0">
-        <v>218.37773606117355</v>
+        <v>287.7949026679911</v>
       </c>
       <c r="B155" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.474177831930916</v>
       </c>
       <c r="C155" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.98486865233469</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="0">
-        <v>218.95858242895315</v>
+        <v>288.43455450946863</v>
       </c>
       <c r="B156" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.474177831930916</v>
       </c>
       <c r="C156" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.944602590540839</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="0">
-        <v>219.53942879673281</v>
+        <v>289.0742063509461</v>
       </c>
       <c r="B157" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.321187259000524</v>
       </c>
       <c r="C157" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.760835467817017</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="0">
-        <v>220.12027516451244</v>
+        <v>289.71385819242357</v>
       </c>
       <c r="B158" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.321187259000524</v>
       </c>
       <c r="C158" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.715511743823306</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="0">
-        <v>220.70112153229206</v>
+        <v>290.3535100339011</v>
       </c>
       <c r="B159" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.235876082695363</v>
       </c>
       <c r="C159" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.700259796230384</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="0">
-        <v>221.28196790007172</v>
+        <v>290.99316187537863</v>
       </c>
       <c r="B160" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.19311442685742</v>
       </c>
       <c r="C160" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.660226897068554</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="0">
-        <v>221.86281426785132</v>
+        <v>291.63281371685611</v>
       </c>
       <c r="B161" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.101727485852329</v>
       </c>
       <c r="C161" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.641699671495516</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="0">
-        <v>222.44366063563098</v>
+        <v>292.27246555833358</v>
       </c>
       <c r="B162" s="0">
-        <v>1.2040200158019487</v>
+        <v>46.052372260298526</v>
       </c>
       <c r="C162" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.528358374330679</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="0">
-        <v>223.0245070034106</v>
+        <v>292.91211739981111</v>
       </c>
       <c r="B163" s="0">
-        <v>1.2040200158019487</v>
+        <v>45.947930929156584</v>
       </c>
       <c r="C163" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.528358374330679</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="0">
-        <v>223.60535337119023</v>
+        <v>293.55176924128858</v>
       </c>
       <c r="B164" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.923528533162902</v>
       </c>
       <c r="C164" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.450045188543946</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="0">
-        <v>224.18619973896989</v>
+        <v>294.19142108276606</v>
       </c>
       <c r="B165" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.905412012979497</v>
       </c>
       <c r="C165" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.450045188543946</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="0">
-        <v>224.76704610674952</v>
+        <v>294.83107292424359</v>
       </c>
       <c r="B166" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.778116010861098</v>
       </c>
       <c r="C166" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.346558944333879</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="0">
-        <v>225.34789247452915</v>
+        <v>295.47072476572106</v>
       </c>
       <c r="B167" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.707461386572483</v>
       </c>
       <c r="C167" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.346558944333879</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0">
-        <v>225.92873884230877</v>
+        <v>296.11037660719859</v>
       </c>
       <c r="B168" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.707461386572483</v>
       </c>
       <c r="C168" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.346558944333879</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="0">
-        <v>226.5095852100884</v>
+        <v>296.75002844867606</v>
       </c>
       <c r="B169" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.64343892317418</v>
       </c>
       <c r="C169" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.267733868895761</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="0">
-        <v>227.09043157786806</v>
+        <v>297.38968029015359</v>
       </c>
       <c r="B170" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.558668743732284</v>
       </c>
       <c r="C170" s="0">
-        <v>0.89348167075665685</v>
+        <v>44.267733868895761</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="0">
-        <v>227.67127794564766</v>
+        <v>298.02933213163107</v>
       </c>
       <c r="B171" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.456803041242509</v>
       </c>
       <c r="C171" s="0">
-        <v>0.81549955182716749</v>
+        <v>44.228964144794048</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="0">
-        <v>228.25212431342732</v>
+        <v>298.6689839731086</v>
       </c>
       <c r="B172" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.456803041242509</v>
       </c>
       <c r="C172" s="0">
-        <v>0.81549955182716749</v>
+        <v>44.205956298580475</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="0">
-        <v>228.83297068120694</v>
+        <v>299.30863581458607</v>
       </c>
       <c r="B173" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.366832910709654</v>
       </c>
       <c r="C173" s="0">
-        <v>0.81549955182716749</v>
+        <v>44.205956298580475</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="0">
-        <v>229.41381704898657</v>
+        <v>299.9482876560636</v>
       </c>
       <c r="B174" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.323959949475963</v>
       </c>
       <c r="C174" s="0">
-        <v>0.73728753826536431</v>
+        <v>44.205956298580475</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="0">
-        <v>229.99466341676623</v>
+        <v>300.58793949754107</v>
       </c>
       <c r="B175" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.256464665254995</v>
       </c>
       <c r="C175" s="0">
-        <v>0.73728753826536431</v>
+        <v>44.105563830704945</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0">
-        <v>230.57550978454583</v>
+        <v>301.22759133901855</v>
       </c>
       <c r="B176" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.223120576169386</v>
       </c>
       <c r="C176" s="0">
-        <v>0.73728753826536431</v>
+        <v>44.105563830704945</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="0">
-        <v>231.15635615232549</v>
+        <v>301.86724318049608</v>
       </c>
       <c r="B177" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.223120576169386</v>
       </c>
       <c r="C177" s="0">
-        <v>0.64694293160270078</v>
+        <v>43.721144925846595</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="0">
-        <v>231.73720252010512</v>
+        <v>302.50689502197355</v>
       </c>
       <c r="B178" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.150011273083671</v>
       </c>
       <c r="C178" s="0">
-        <v>0.64694293160270078</v>
+        <v>43.721144925846595</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="0">
-        <v>232.31804888788474</v>
+        <v>303.14654686345102</v>
       </c>
       <c r="B179" s="0">
-        <v>1.1638860152752171</v>
+        <v>45.039376841040408</v>
       </c>
       <c r="C179" s="0">
-        <v>0.64694293160270078</v>
+        <v>43.689666630582281</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="0">
-        <v>232.8988952556644</v>
+        <v>303.78619870492855</v>
       </c>
       <c r="B180" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.99879662198515</v>
       </c>
       <c r="C180" s="0">
-        <v>0.64694293160270078</v>
+        <v>43.621110935825712</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="0">
-        <v>233.479741623444</v>
+        <v>304.42585054640608</v>
       </c>
       <c r="B181" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.927750562362235</v>
       </c>
       <c r="C181" s="0">
-        <v>0.64694293160270078</v>
+        <v>43.5446166734598</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="0">
-        <v>234.06058799122366</v>
+        <v>305.06550238788356</v>
       </c>
       <c r="B182" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.903150964404375</v>
       </c>
       <c r="C182" s="0">
-        <v>0.64694293160270078</v>
+        <v>43.457619645168521</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="0">
-        <v>234.64143435900329</v>
+        <v>305.70515422936103</v>
       </c>
       <c r="B183" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.859303281337219</v>
       </c>
       <c r="C183" s="0">
-        <v>0.62044394979340622</v>
+        <v>43.457619645168521</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="0">
-        <v>235.22228072678291</v>
+        <v>306.34480607083856</v>
       </c>
       <c r="B184" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.816420722643016</v>
       </c>
       <c r="C184" s="0">
-        <v>0.62044394979340622</v>
+        <v>43.391663288392493</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="0">
-        <v>235.80312709456254</v>
+        <v>306.98445791231603</v>
       </c>
       <c r="B185" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.816420722643016</v>
       </c>
       <c r="C185" s="0">
-        <v>0.62044394979340622</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="0">
-        <v>236.38397346234217</v>
+        <v>307.62410975379351</v>
       </c>
       <c r="B186" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.816420722643016</v>
       </c>
       <c r="C186" s="0">
-        <v>0.62044394979340622</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="0">
-        <v>236.96481983012183</v>
+        <v>308.26376159527104</v>
       </c>
       <c r="B187" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.816420722643016</v>
       </c>
       <c r="C187" s="0">
-        <v>0.62044394979340622</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="0">
-        <v>237.54566619790143</v>
+        <v>308.90341343674851</v>
       </c>
       <c r="B188" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.760235547813522</v>
       </c>
       <c r="C188" s="0">
-        <v>0.58151803673983937</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="0">
-        <v>238.12651256568108</v>
+        <v>309.54306527822604</v>
       </c>
       <c r="B189" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.760235547813522</v>
       </c>
       <c r="C189" s="0">
-        <v>0.58151803673983937</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="0">
-        <v>238.70735893346071</v>
+        <v>310.18271711970351</v>
       </c>
       <c r="B190" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.760235547813522</v>
       </c>
       <c r="C190" s="0">
-        <v>0.58151803673983937</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="0">
-        <v>239.28820530124034</v>
+        <v>310.82236896118104</v>
       </c>
       <c r="B191" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.544310754877031</v>
       </c>
       <c r="C191" s="0">
-        <v>0.58151803673983937</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="0">
-        <v>239.86905166902</v>
+        <v>311.46202080265851</v>
       </c>
       <c r="B192" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.544310754877031</v>
       </c>
       <c r="C192" s="0">
-        <v>0.58151803673983937</v>
+        <v>43.349036458605042</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="0">
-        <v>240.4498980367996</v>
+        <v>312.10167264413599</v>
       </c>
       <c r="B193" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.361321921698149</v>
       </c>
       <c r="C193" s="0">
-        <v>0.55666034616594462</v>
+        <v>43.14390677886405</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="0">
-        <v>241.03074440457925</v>
+        <v>312.74132448561352</v>
       </c>
       <c r="B194" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.238932476798077</v>
       </c>
       <c r="C194" s="0">
-        <v>0.55666034616594462</v>
+        <v>43.14390677886405</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="0">
-        <v>241.61159077235891</v>
+        <v>313.38097632709099</v>
       </c>
       <c r="B195" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.218472031530439</v>
       </c>
       <c r="C195" s="0">
-        <v>0.55666034616594462</v>
+        <v>42.893613195663669</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="0">
-        <v>242.19243714013851</v>
+        <v>314.02062816856852</v>
       </c>
       <c r="B196" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.218472031530439</v>
       </c>
       <c r="C196" s="0">
-        <v>0.55666034616594462</v>
+        <v>42.874461032444984</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="0">
-        <v>242.77328350791817</v>
+        <v>314.660280010046</v>
       </c>
       <c r="B197" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.218472031530439</v>
       </c>
       <c r="C197" s="0">
-        <v>0.53011108574208588</v>
+        <v>42.874461032444984</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="0">
-        <v>243.35412987569779</v>
+        <v>315.29993185152352</v>
       </c>
       <c r="B198" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.150815205400221</v>
       </c>
       <c r="C198" s="0">
-        <v>0.53011108574208588</v>
+        <v>42.8267873909369</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="0">
-        <v>243.93497624347742</v>
+        <v>315.939583693001</v>
       </c>
       <c r="B199" s="0">
-        <v>1.1638860152752171</v>
+        <v>44.031732522820804</v>
       </c>
       <c r="C199" s="0">
-        <v>0.53011108574208588</v>
+        <v>42.8267873909369</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="0">
-        <v>244.51582261125708</v>
+        <v>316.57923553447847</v>
       </c>
       <c r="B200" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.946160703499992</v>
       </c>
       <c r="C200" s="0">
-        <v>0.53011108574208588</v>
+        <v>42.723678704432935</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="0">
-        <v>245.09666897903668</v>
+        <v>317.218887375956</v>
       </c>
       <c r="B201" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.946160703499992</v>
       </c>
       <c r="C201" s="0">
-        <v>0.53011108574208588</v>
+        <v>42.68008659522161</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="0">
-        <v>245.67751534681634</v>
+        <v>317.85853921743347</v>
       </c>
       <c r="B202" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.946160703499992</v>
       </c>
       <c r="C202" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.614427862889436</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="0">
-        <v>246.25836171459596</v>
+        <v>318.498191058911</v>
       </c>
       <c r="B203" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.946160703499992</v>
       </c>
       <c r="C203" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.579656844712396</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="0">
-        <v>246.83920808237559</v>
+        <v>319.13784290038848</v>
       </c>
       <c r="B204" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.771731135452725</v>
       </c>
       <c r="C204" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.538175533258041</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0">
-        <v>247.42005445015522</v>
+        <v>319.77749474186601</v>
       </c>
       <c r="B205" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.743994019690206</v>
       </c>
       <c r="C205" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.538175533258041</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="0">
-        <v>248.00090081793485</v>
+        <v>320.41714658334348</v>
       </c>
       <c r="B206" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.743994019690206</v>
       </c>
       <c r="C206" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.461658440461605</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0">
-        <v>248.58174718571451</v>
+        <v>321.05679842482095</v>
       </c>
       <c r="B207" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.696130812437311</v>
       </c>
       <c r="C207" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.461658440461605</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="0">
-        <v>249.16259355349411</v>
+        <v>321.69645026629849</v>
       </c>
       <c r="B208" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.696130812437311</v>
       </c>
       <c r="C208" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.418956084148363</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0">
-        <v>249.74343992127376</v>
+        <v>322.33610210777596</v>
       </c>
       <c r="B209" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.581279081216437</v>
       </c>
       <c r="C209" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.384247457501615</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="0">
-        <v>250.32428628905339</v>
+        <v>322.97575394925349</v>
       </c>
       <c r="B210" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.567829647931902</v>
       </c>
       <c r="C210" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.348675273843256</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0">
-        <v>250.90513265683302</v>
+        <v>323.61540579073096</v>
       </c>
       <c r="B211" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.517205457674017</v>
       </c>
       <c r="C211" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.290737700880499</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="0">
-        <v>251.48597902461267</v>
+        <v>324.25505763220849</v>
       </c>
       <c r="B212" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.42116676831256</v>
       </c>
       <c r="C212" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.290737700880499</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="0">
-        <v>252.06682539239228</v>
+        <v>324.89470947368596</v>
       </c>
       <c r="B213" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.401342595431011</v>
       </c>
       <c r="C213" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.245047532223907</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="0">
-        <v>252.64767176017193</v>
+        <v>325.53436131516344</v>
       </c>
       <c r="B214" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.364747085495502</v>
       </c>
       <c r="C214" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.155455272151045</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0">
-        <v>253.22851812795156</v>
+        <v>326.17401315664097</v>
       </c>
       <c r="B215" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.364747085495502</v>
       </c>
       <c r="C215" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.109058958476339</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0">
-        <v>253.80936449573119</v>
+        <v>326.81366499811844</v>
       </c>
       <c r="B216" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.243637635344896</v>
       </c>
       <c r="C216" s="0">
-        <v>0.50342680019519315</v>
+        <v>42.109058958476339</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="0">
-        <v>254.39021086351085</v>
+        <v>327.45331683959591</v>
       </c>
       <c r="B217" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.243637635344896</v>
       </c>
       <c r="C217" s="0">
-        <v>0.46457665398900805</v>
+        <v>42.02219160582785</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0">
-        <v>254.97105723129044</v>
+        <v>328.09296868107344</v>
       </c>
       <c r="B218" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.191042001786357</v>
       </c>
       <c r="C218" s="0">
-        <v>0.46457665398900805</v>
+        <v>42.02219160582785</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="0">
-        <v>255.5519035990701</v>
+        <v>328.73262052255097</v>
       </c>
       <c r="B219" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.114915871805252</v>
       </c>
       <c r="C219" s="0">
-        <v>0.46457665398900805</v>
+        <v>42.02219160582785</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0">
-        <v>256.1327499668497</v>
+        <v>329.37227236402845</v>
       </c>
       <c r="B220" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.114915871805252</v>
       </c>
       <c r="C220" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.98473521634682</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="0">
-        <v>256.71359633462936</v>
+        <v>330.01192420550592</v>
       </c>
       <c r="B221" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.059560946928954</v>
       </c>
       <c r="C221" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.98473521634682</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0">
-        <v>257.29444270240902</v>
+        <v>330.65157604698345</v>
       </c>
       <c r="B222" s="0">
-        <v>1.1638860152752171</v>
+        <v>43.028174870729444</v>
       </c>
       <c r="C222" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.88062327610227</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0">
-        <v>257.87528907018861</v>
+        <v>331.29122788846092</v>
       </c>
       <c r="B223" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.931978887572896</v>
       </c>
       <c r="C223" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.88062327610227</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="0">
-        <v>258.45613543796827</v>
+        <v>331.9308797299384</v>
       </c>
       <c r="B224" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.931978887572896</v>
       </c>
       <c r="C224" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.865381524266276</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="0">
-        <v>259.03698180574793</v>
+        <v>332.57053157141593</v>
       </c>
       <c r="B225" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.931978887572896</v>
       </c>
       <c r="C225" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.816009698314304</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="0">
-        <v>259.61782817352753</v>
+        <v>333.2101834128934</v>
       </c>
       <c r="B226" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.931978887572896</v>
       </c>
       <c r="C226" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.816009698314304</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="0">
-        <v>260.19867454130713</v>
+        <v>333.84983525437087</v>
       </c>
       <c r="B227" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.866110420106338</v>
       </c>
       <c r="C227" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.774424312537306</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0">
-        <v>260.77952090908678</v>
+        <v>334.4894870958484</v>
       </c>
       <c r="B228" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.794339333910926</v>
       </c>
       <c r="C228" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.774424312537306</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="0">
-        <v>261.36036727686644</v>
+        <v>335.12913893732593</v>
       </c>
       <c r="B229" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.700355930745438</v>
       </c>
       <c r="C229" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.647290893717454</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="0">
-        <v>261.94121364464604</v>
+        <v>335.76879077880341</v>
       </c>
       <c r="B230" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.700355930745438</v>
       </c>
       <c r="C230" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.647290893717454</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0">
-        <v>262.5220600124257</v>
+        <v>336.40844262028088</v>
       </c>
       <c r="B231" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.633486000703989</v>
       </c>
       <c r="C231" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.60903440761696</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="0">
-        <v>263.10290638020535</v>
+        <v>337.04809446175841</v>
       </c>
       <c r="B232" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.592175252153076</v>
       </c>
       <c r="C232" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.60903440761696</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="0">
-        <v>263.68375274798496</v>
+        <v>337.68774630323594</v>
       </c>
       <c r="B233" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.592175252153076</v>
       </c>
       <c r="C233" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.60903440761696</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="0">
-        <v>264.26459911576461</v>
+        <v>338.32739814471336</v>
       </c>
       <c r="B234" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.592175252153076</v>
       </c>
       <c r="C234" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.563871406526417</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="0">
-        <v>264.84544548354421</v>
+        <v>338.96704998619089</v>
       </c>
       <c r="B235" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.54565755403533</v>
       </c>
       <c r="C235" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.536294708917581</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="0">
-        <v>265.42629185132387</v>
+        <v>339.60670182766842</v>
       </c>
       <c r="B236" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.491422393459033</v>
       </c>
       <c r="C236" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.518840232430506</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="0">
-        <v>266.00713821910347</v>
+        <v>340.24635366914595</v>
       </c>
       <c r="B237" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.491422393459033</v>
       </c>
       <c r="C237" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.518840232430506</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="0">
-        <v>266.58798458688312</v>
+        <v>340.88600551062336</v>
       </c>
       <c r="B238" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.330940741061085</v>
       </c>
       <c r="C238" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.518840232430506</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="0">
-        <v>267.16883095466278</v>
+        <v>341.52565735210089</v>
       </c>
       <c r="B239" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.330940741061085</v>
       </c>
       <c r="C239" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.453833454694063</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="0">
-        <v>267.74967732244238</v>
+        <v>342.16530919357842</v>
       </c>
       <c r="B240" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.261729054954714</v>
       </c>
       <c r="C240" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.416614807624242</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="0">
-        <v>268.33052369022209</v>
+        <v>342.80496103505584</v>
       </c>
       <c r="B241" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.261729054954714</v>
       </c>
       <c r="C241" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.416614807624242</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="0">
-        <v>268.91137005800169</v>
+        <v>343.44461287653337</v>
       </c>
       <c r="B242" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.226286527241946</v>
       </c>
       <c r="C242" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.279022092261513</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="0">
-        <v>269.49221642578129</v>
+        <v>344.0842647180109</v>
       </c>
       <c r="B243" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.226286527241946</v>
       </c>
       <c r="C243" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="0">
-        <v>270.07306279356095</v>
+        <v>344.72391655948837</v>
       </c>
       <c r="B244" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.208574079098582</v>
       </c>
       <c r="C244" s="0">
-        <v>0.46457665398900805</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="0">
-        <v>270.65390916134061</v>
+        <v>345.36356840096585</v>
       </c>
       <c r="B245" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.170298566099291</v>
       </c>
       <c r="C245" s="0">
-        <v>0.41336063058533684</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="0">
-        <v>271.23475552912021</v>
+        <v>346.00322024244338</v>
       </c>
       <c r="B246" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.05082911684633</v>
       </c>
       <c r="C246" s="0">
-        <v>0.41336063058533684</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="0">
-        <v>271.81560189689986</v>
+        <v>346.64287208392091</v>
       </c>
       <c r="B247" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.05082911684633</v>
       </c>
       <c r="C247" s="0">
-        <v>0.41336063058533684</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0">
-        <v>272.39644826467946</v>
+        <v>347.28252392539838</v>
       </c>
       <c r="B248" s="0">
-        <v>1.1638860152752171</v>
+        <v>42.05082911684633</v>
       </c>
       <c r="C248" s="0">
-        <v>0.41336063058533684</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="0">
-        <v>272.97729463245912</v>
+        <v>347.92217576687585</v>
       </c>
       <c r="B249" s="0">
-        <v>1.1638860152752171</v>
+        <v>41.970519925325817</v>
       </c>
       <c r="C249" s="0">
-        <v>0.41336063058533684</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0">
-        <v>273.55814100023872</v>
+        <v>348.56182760835338</v>
       </c>
       <c r="B250" s="0">
-        <v>1.1638860152752171</v>
+        <v>41.891636464740877</v>
       </c>
       <c r="C250" s="0">
-        <v>0.41336063058533684</v>
+        <v>41.193186380066464</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="0">
-        <v>274.13898736801838</v>
+        <v>349.20147944983086</v>
       </c>
       <c r="B251" s="0">
-        <v>1.1638860152752171</v>
+        <v>41.891636464740877</v>
       </c>
       <c r="C251" s="0">
-        <v>0.386565828728068</v>
+        <v>41.017213187273882</v>
       </c>
     </row>
   </sheetData>

</xml_diff>